<commit_message>
Finalize Iteration 3 - website content scraping and integration into GPT for all companies
</commit_message>
<xml_diff>
--- a/GPT_Responses_Iteration3.xlsx
+++ b/GPT_Responses_Iteration3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>Not Comparable.
-While both companies operate in the logistics industry, the core functions and target industries of the two companies differ significantly. The tested party in the medical industry coordinates shipments for Africa, while the company under review provides general logistics services across various industries in Bulgaria. The services offered, target markets, and overall business focus are not directly comparable for transfer pricing purposes.</t>
+Although both companies operate in the logistics and transportation industry, the specific functions and services offered by the company under review, A LOGISTICS EOOD, seem to be more focused on general logistics and supply chain solutions for various industries. In contrast, the tested party in the medical industry in Africa specializes in procurement and logistics services, specifically coordinating shipments, handling local storage, and overseeing delivery processes. The differences in their core functions and target industries make them not directly comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -490,8 +490,361 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>Comparable
+Both companies are involved in the transportation and logistics industry, providing services related to cargo shipments and handling. While the tested party focuses on medical industry logistics in Africa, the company under review specializes in international freight forwarding and cargo transportation services in Hungary. The core functions and services offered by both companies align closely, making them comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: ALB - AREA LOGISTICA DA BOBADELA, S.A.
+Country: Portugal
+Industry: 4789 - Trans: Transportation Services, nec
+Description: This company operates within the logistics sector, specializing in warehouse management and distribution services. It caters to a diverse customer base, including businesses seeking efficient supply chain solutions. 
+Website: www.alb.com.pt
+Website Content Extracted:
+ Error accessing website: http://www.alb.com.pt – HTTPConnectionPool(host='www.alb.com.pt', port=80): Max retries exceeded with url: / (Caused by NameResolutionError("&lt;urllib3.connection.HTTPConnection object at 0x7f617ce0e090&gt;: Failed to resolve 'www.alb.com.pt' ([Errno -2] Name or service not known)"))
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Not Comparable.
+The company under review operates in the logistics sector, specializing in warehouse management and distribution services, catering to businesses seeking supply chain solutions. On the other hand, the tested party in the medical industry focuses on procurement and logistics services, coordinating shipments and overseeing delivery processes in Africa. The core functions and industries of these two companies are quite different, making them not comparable for transfer pricing purposes. Additionally, the website was inaccessible, which limits the information available for comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: ALBERTS LOGISTIK GMBH &amp; CO. KG
+Country: Germany
+Industry: 4789 - Trans: Transportation Services, nec
+Description: The company provides transportation, warehousing, and inventory management services, catering to manufacturers, distributors, and retailers within the region and beyond
+Website: WWW.ALBERTS.DE
+Website Content Extracted:
+Alberts - Gemacht, um zu halten. - Alberts Zum Haupt-Inhalt Menü Alberts search Produkte Produkte Produkte Überblick ansehen Eisenwaren Zauntechnik Profile &amp; Bleche Weitere Produkte Magazin Unternehmen Unternehmen Unternehmen Überblick ansehen Über uns Geschichte Werte und Ziele Qualität und Umwelt Made in Herscheid Alberts Gruppe Messen Lösungen Lösungen Lösungen Überblick ansehen Heimwerker Handwerker Händler Industrieservice Service Service Service Überblick ansehen Kontakt Ansprechpartner Bestellung Ersatzteile Downloads Karriere Karriere Karriere Überblick ansehen Arbeiten bei Alberts Hand in Hand Stellen- &amp; Ausbildungsangebote Ausbildung Duales Studium  de en English fr Français it Italiano es Español pl Polski Händler-Login Alles aus Eisen Alles aus Eisen Unsere Eisenwaren sind Problemlöser in Spitzenqualität. Produkte ansehen Aus Liebe zum Zaun Aus Liebe zum Zaun Hochwertige Zaunsysteme für jeden Einsatzbereich. Produkte ansehen Profis für Profile Profis für Profile Ein umfang
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Not Comparable 
+The company under review, ALBERTS LOGISTIK GMBH &amp; CO. KG, is primarily focused on providing transportation, warehousing, and inventory management services in the region, catering to manufacturers, distributors, and retailers. On the other hand, the tested party is a procurement and logistics service provider in the medical industry in the Netherlands, with a focus on coordinating shipments, handling local storage, and overseeing delivery processes in Africa. There are significant differences in the core functions, industry focus, and geographic scope between the two companies, making them not comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: ALC AUTOMOTIVE LOGISTIC CENTER GMBH
+Country: Germany
+Industry: 7699 - Serv: Repair Services, nec
+Description: The company provides specialized logistics services for automotive manufacturers and suppliers, focusing on efficient distribution, storage, and transportation of automotive parts and vehicles. The customer base primarily includes automotive manufacturers and suppliers
+Website: WWW.ALC-LOGISTIC.DE
+Website Content Extracted:
+ALC AUTOMOTIVE LOGISTIC CENTER Home Über Uns Leistungen Automotive Logistik Werkslogistik Distributionslogistik Referenzen Jobs Kontakt × Home Über Uns Leistungen Referenzen Jobs Kontakt 01 Automotive Logistic Center ALC AUTOMOTIVE LOGISTIC CENTER Wir sind ein mittelständisches familiengeführtes Unternehmen mit Spezialisierung auf Dienstleistungen in den Bereichen Automotive Logistik, Werkslogistik und Distributionslogistik. 02 Über Uns Die Gründung unseres traditionsreichen Familienunternehmens geht auf 1853 zurück. Eine Zusammenarbeit mit der Automobil-Industrie begann mit der Herstellung von Exportverpackungen und Versandbehältern. Später wurden mit dem selbstentwickelten Werkstoff Schollit© Karosserieteile hergestellt. Mehr Über Uns 03 Leistungen 200 Mitarbeiter im Bereich Automotive Logistik, Werkslogistik &amp; Distributionslogistik. Alle Leistungen 04 Referenzen Unsere Kunden schätzen besonders unsere Flexibilität bei der Umsetzung von Logistikprojekten. Alle Referenzen 05 Jobs Aktu
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Comparable
+Both companies provide logistics services within their respective industries, focusing on coordination, storage, and transportation of goods. While the tested party operates in the medical industry and the company under review operates in the automotive industry, the core functions and services offered by both companies are similar enough to be considered comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: ALFA SHIPPING AGENCY SRL
+Country: Italy
+Industry: 4789 - Trans: Transportation Services, nec
+Description: The company specializes in providing services related to shipping and maritime logistics. Its primary offerings include port agency services, cargo handling, and maritime consultancy.
+Website: WWW.ALFASHIPPING.IT
+Website Content Extracted:
+ALFA SHIPPING s.r.l. Toggle navigation Home Agency Chartering Contact Since 1998, the same passion for shipping. Alfa Shipping Alfa Shipping Agency Srl was founded in 1998 in order to support one of the major terminals in Porto Marghera, Italy.During the years, except from being involved as shipping agency , we also specialized as brokers , both part and full charter for all kind of commodities, but mainly within project cargo to and from/to worldwide destinations. Experience and new ideas We have long experience in project cargoes and heavy-lift transportation , with more than 30 years behind us in this field. In June 2014 Mr. Stefano Lanata, who is working in this kind of business from more than 10 years, joined us with the aim to improve our activities. Great partnerships, low rates Currently we are offering our assistance to several forwarding companies within the project trade and we have very good and close relationship with several Shipping Companies and with some of the major h
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Comparable.
+Both companies are involved in providing logistics and shipping-related services, with a focus on coordinating shipments and overseeing delivery processes. While the industries may differ slightly, the core functions and services offered by both companies are similar enough to be considered comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: ALMEIDA &amp; PESTANA, LDA
+Country: Portugal
+Industry: 4789 - Trans: Transportation Services, nec
+Description: This company specializes in providing tailored products and services across various sectors, catering primarily to local and regional customers
+Website: WWW.ALMEIDAPESTANA.PT
+Website Content Extracted:
+ Error accessing website: http://WWW.ALMEIDAPESTANA.PT – HTTPConnectionPool(host='www.almeidapestana.pt', port=80): Max retries exceeded with url: / (Caused by NameResolutionError("&lt;urllib3.connection.HTTPConnection object at 0x7f617cbff3d0&gt;: Failed to resolve 'www.almeidapestana.pt' ([Errno -2] Name or service not known)"))
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Not Comparable.
 Reasoning:
-Both the tested party and the company under review are involved in logistics services, with a focus on international freight forwarding and cargo transportation. They cater to businesses in need of efficient logistics solutions, which makes them comparable for transfer pricing purposes.</t>
+The company under review, ALMEIDA &amp; PESTANA, LDA, operates in the transportation services industry in Portugal, providing tailored products and services to local and regional customers. This is different from the tested party, a procurement and logistics service provider in the medical industry in the Netherlands. The core functions and industries of the two companies are not sufficiently similar to be considered comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: ALOG LTD OOD
+Country: Bulgaria
+Industry: 4789 - Trans: Transportation Services, nec
+Description: The company operates from a modest facility in this locality, specializing in providing tailored services to its clientele
+Website: WWW.ALOG-BG.COM
+Website Content Extracted:
+Начало - Александър Логистикс (Alexander Logistics) Начало За нас Услуги Автомобилен транспорт Вътрешен дистрибуция Въздушен транспорт Морски транспорт Складова логистика Митнически услуги Блог Новини Контакти 0700 50 577 Запитване 0700 50 577 Начало За нас Услуги Автомобилен транспорт Вътрешен дистрибуция Въздушен транспорт Морски транспорт Складова логистика Митнически услуги Блог Новини Контакти 0700 50 577 Запитване Начало Александър Логистикс e частна компания, управлявана от собствениците, споделяйки философията, че бъдещето принадлежи на иновациите, гъвкавостта и екипната работа. Способността за създаване на партньорства и работа в мрежи е ключов фактор за изграждане на успешни вериги на доставките. Повече за нас Автомобилен транспорт Въздушен транспорт Морски транспорт Складова логистика Митнически услуги Онлайн услуги Клиентски портал Информация за фактура Проследяване на пратка Партньорски портал Нов акаунт Новини | 01/29/25 10:36 AM Модерна складова база… „Александър Логисти
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Not Comparable
+Reasoning:
+The company under review, ALOG LTD OOD, operates in the transportation industry in Bulgaria, offering services such as automotive transport, air transport, sea transport, and warehouse logistics. The tested party is a procurement and logistics service provider in the medical industry in the Netherlands, focused on coordinating shipments, handling local storage, and overseeing delivery processes in Africa. The industries, functions, and geographic locations of the two companies are significantly different, making them not comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: AUTOTALLERES GUTIERREZ SL
+Country: Spain
+Industry: 7699 - Serv: Repair Services, nec
+Description: Specializes in automobile repair and maintenance services. Its headquarters is equipped with advanced tools and facilities, catering to a local customer base that includes individual vehicle owners and businesses.
+Website: WWW.TALLERESGUTIERREZ.ES
+Website Content Extracted:
+Talleres Gutierrez Valencia Web en Construcción
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Not Comparable.
+The company under review, AUTOTALLERES GUTIERREZ SL, specializes in automobile repair and maintenance services, while the tested party is a procurement and logistics service provider in the medical industry. These two companies operate in completely different industries and have different core functions, making them not comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: B.T.L. TRANSPORT LOGISTICS S.A.
+Country: Greece
+Industry: 4789 - Trans: Transportation Services, nec
+Description: The company specializes in providing a wide range of logistics services, including freight transportation, warehousing, and supply chain management solutions
+Website: WWW.BTLSA.GR
+Website Content Extracted:
+ Unable to retrieve content from website: http://WWW.BTLSA.GR
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Not Comparable.
+While both companies operate in the logistics industry, the tested party specifically focuses on procurement and logistics services in the medical industry in Africa, while the company under review offers a wider range of logistics services in Greece. The differences in geographic focus, industry specialization, and core functions indicate that these companies may not be directly comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: BARBIERI GESTIONI SRL
+Country: Italy
+Industry: 4789 - Trans: Transportation Services, nec
+Description: The company focuses on providing management and administrative services tailored to its clients' needs.
+Website: WWW.BARBIERITRASPORTI.IT
+Website Content Extracted:
+ Unable to retrieve content from website: http://WWW.BARBIERITRASPORTI.IT
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Not Comparable.
+Reasoning: The tested party is a procurement and logistics service provider in the medical industry, while the company under review focuses on providing management and administrative services in the transportation industry. The differences in core functions and industries make these companies not comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: BARTRANSIS UAB
+Country: Lithuania
+Industry: 4789 - Trans: Transportation Services, nec
+Description: the firm likely caters to regional or international customers across diverse sectors
+Website: WWW.BARTRANSIS.LT
+Website Content Extracted:
+ Unable to retrieve content from website: http://WWW.BARTRANSIS.LT
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Not Comparable
+Reasoning:
+The limited information available about BARTRANSIS UAB, coupled with the lack of website content, makes it difficult to assess if this company is truly comparable for transfer pricing purposes. Additionally, the specific industry focus and core functions of the tested party in the medical procurement and logistics sector may not align with the transportation services sector that BARTRANSIS UAB operates in. Without more detailed information, it is challenging to determine if the two companies are truly comparable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: BELLANDI SRL
+Country: Italy
+Industry: 4499 - Trans: Water Transportation Services, nec
+Description: Retail-boats and marine supplies
+Website: WWW.BARCHEBELLANDI.COM
+Website Content Extracted:
+CONCESSIONARIO UFFICIALE BENETEAU - DEALER BENETEAU - BELLANDI SRL Salta al contenuto Home I nostri servizi Espandi Vendita Nuovo/Usato Espandi Concessionario Beneteau Maxima Boats Punto vendita accessori Assistenza Marina Noleggio Espandi Noleggio barche Desenzano Vendita Nuovo/Usato Chi siamo Espandi L’azienda Contatti Come raggiungerci Orari di apertura Staff Dicono di noi Barchemania Blog Lavora con noi Attiva/disattiva menu Slide 1 Slide 2 Slide 7 Slide 3 Slide 4 Slide 8 Slide 5 Slide 6 Concessionario BENETEAU Barche Bellandi è partner del marchio BENETEAU, azienda francese che produce imbarcazioni da diporto tra cui barche a vela e motoryacht. Fondata nel 1884, l’azienda è una delle più grandi e storiche del mondo della produzione di imbarcazioni. La loro attenzione al design, alla qualità costruttiva e all’innovazione li rende una scelta prestigiosa per i diportisti di tutto il mondo. Rivolgiti a noi se cerchi un partner qualificato nella vendita di barche Beneteau. Barche Bella
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Not Comparable.
+The company under review, BELLANDI SRL, operates in the retail-boats and marine supplies industry, specifically in water transportation services. Their core business activities do not align with the procurement and logistics services provided by the tested party in the medical industry. Additionally, the geographical focus and customer base of the two companies differ significantly. As a result, they are not comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: BEST LOGISTICS NORTH S.A.
+Country: Greece
+Industry: 4789 - Trans: Transportation Services, nec
+Description: specializes in providing logistics and transportation services. Its core offerings include freight forwarding, customs brokerage, warehouse management, and third-party logistics solutions
+Website: WWW.BESTLOGISTICS-NORTH.GR
+Website Content Extracted:
+Αρχική - Best Logistics North Μετάβαση στο περιεχόμενο Αναζήτηση για: Αναζήτηση Αρχική Σχετικά με εμάς Υπηρεσίες Εναλλαγή μενού Οδική μεταφορά Συνδυασμένη μεταφορά (με τρένο) Θαλάσσια μεταφορά Εσωτερική διανομή &amp; αποθήκευση Ασφάλιση Μεταφοράς Logistics Τα νέα μας Επικοινωνία Ελληνικά Εναλλαγή μενού English Deutsch Français Main Menu Search for: Αρχική Σχετικά με εμάς Υπηρεσίες Εναλλαγή μενού Οδική μεταφορά Συνδυασμένη μεταφορά (με τρένο) Θαλάσσια Μεταφορά Εσωτερική διανομή &amp; αποθήκευση Ασφάλιση Μεταφοράς Logistics Τα νέα μας Επικοινωνία English Deutsch Ελληνικά Français Οι μεταφορές είναι το πάθος μας Περισσότερα Γιατί με τη Best Logistics North SA; Your Path to the Best Logistics Solutions Εξαιρετική εξυπηρέτηση Είμαστε υπερήφανοι για την παροχή εξαιρετικών υπηρεσιών στους πελάτες μας. Δίνουμε προτεραιότητα στην ικανοποίηση των πελατών και κάνουμε το καλύτερο δυνατό για να διασφαλίσουμε ότι όλες οι ανάγκες σας για μεταφορά θα ικανοποιηθούν με τον μέγιστο επαγγελματισμό και αποτελεσματ
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Not Comparable.
+While both companies operate in the logistics industry, the core functions and services offered are quite different. The tested party mainly focuses on procurement and logistics services in the medical industry in Africa, while the company under review in Greece specializes in logistics and transportation services, including freight forwarding and customs brokerage. The differences in core functions and target markets make these two companies not comparable for transfer pricing purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Tested Party:
+A Netherlands-based procurement and logistics service provider in the medical industry, functioning as a limited-risk entity. Its core functions include coordinating shipments, handling local storage, and overseeing delivery processes in Africa.
+Company Under Review:
+Name: BI-KA LOGISZTIKA KORLATOLT FELELOSSEGU TARSASAG
+Country: Hungary
+Industry: 4789 - Trans: Transportation Services, nec
+Description: The company operates within the logistics and transportation sector, providing a range of services designed to support supply chain and logistics management.
+Website: WWW.BI-KA.HU
+Website Content Extracted:
+BI-KA Logisztika Kft. - Főoldal BI-KA Logisztika Kft. info@bi-ka.hu +36-56/524-050 Toggle navigation Home About Adatvédelem Ajánlatkérés Ajánlatkérés Gyors ajánlatkérés Részletes ajánlatkérés Aktualitások Állásajánlat: Készletgazda Állásajánlat: nemzetközi fuvarszervező Állásajánlat: Nemzetközi gépjárművezető Állásajánlat: Nemzetközi gépjárművezető FIX körfuvarokra Állásajánlat: Nemzetközi szállítmányozó (Budapest) Alvállalkozóinknak Blog Brexit Cart Checkout Company Contact ENG Fiókom Hasznos Impresszum Megbízóinknak Segédlet árajánlathoz Teendők első fuvar esetén Teendők kár esetén Híreink James Watson Junior Program Kapcsolat Karácsonyi nyereményjáték Koronavírus tájékoztató Kosár Megbízóinknak Agrárpiaci megoldások Ajánlatkérés Bérleti konstrukciók a BI-KA Logisztika ajánlásával Nyomtatványok Raktározás Szaktanácsadás Szállítmánybiztosítás Szállítmányozás Belföldi Nemzetközi TSM információk – össztömeg és tengelysúly Mobilitási csomag My account Nemzetközi gépjárművezető Pályázatok
+Question:
+Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
+Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
+</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Not Comparable
+While both companies operate within the logistics and transportation sector, there are significant differences in their core functions and geographical focus. The tested party is specifically focused on procurement and logistics services in the medical industry in Africa, while the company under review operates in Hungary and offers a range of transportation services. The differing industry focuses and geographical regions make these companies not directly comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Improves webpage speed and adds a user interface
Adds a Streamlit web app interface with file upload and input fields for GPT analysis, addressing user concerns about slow processing and lack of visual feedback.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/GPT_Responses_Iteration3.xlsx
+++ b/GPT_Responses_Iteration3.xlsx
@@ -463,7 +463,7 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>Not Comparable.
-Although both companies operate in the logistics and transportation industry, the specific functions and services offered by the company under review, A LOGISTICS EOOD, seem to be more focused on general logistics and supply chain solutions for various industries. In contrast, the tested party in the medical industry in Africa specializes in procurement and logistics services, specifically coordinating shipments, handling local storage, and overseeing delivery processes. The differences in their core functions and target industries make them not directly comparable for transfer pricing purposes.</t>
+While both companies are involved in logistics and transportation services, the specific functions and industries they specialize in are different. The tested party focuses on procurement and logistics services in the medical industry in Africa, while the company under review offers general logistics and supply chain solutions to businesses across various industries in Bulgaria. The differences in their core functions, target industries, and geographical focus make them not directly comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -489,8 +489,8 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Comparable
-Both companies are involved in the transportation and logistics industry, providing services related to cargo shipments and handling. While the tested party focuses on medical industry logistics in Africa, the company under review specializes in international freight forwarding and cargo transportation services in Hungary. The core functions and services offered by both companies align closely, making them comparable for transfer pricing purposes.</t>
+          <t>Not Comparable.
+While both companies operate in the logistics industry, the tested party specifically focuses on procurement and logistics services in the medical industry, whereas the company under review specializes in international freight forwarding and cargo transportation services for businesses in general. The differences in their core functions and industries make them not directly comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -507,7 +507,7 @@
 Description: This company operates within the logistics sector, specializing in warehouse management and distribution services. It caters to a diverse customer base, including businesses seeking efficient supply chain solutions. 
 Website: www.alb.com.pt
 Website Content Extracted:
- Error accessing website: http://www.alb.com.pt – HTTPConnectionPool(host='www.alb.com.pt', port=80): Max retries exceeded with url: / (Caused by NameResolutionError("&lt;urllib3.connection.HTTPConnection object at 0x7f617ce0e090&gt;: Failed to resolve 'www.alb.com.pt' ([Errno -2] Name or service not known)"))
+ Error accessing website: http://www.alb.com.pt – HTTPConnectionPool(host='www.alb.com.pt', port=80): Max retries exceeded with url: / (Caused by NameResolutionError("&lt;urllib3.connection.HTTPConnection object at 0x7efd723f6dd0&gt;: Failed to resolve 'www.alb.com.pt' ([Errno -2] Name or service not known)"))
 Question:
 Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
 Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
@@ -517,7 +517,8 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>Not Comparable.
-The company under review operates in the logistics sector, specializing in warehouse management and distribution services, catering to businesses seeking supply chain solutions. On the other hand, the tested party in the medical industry focuses on procurement and logistics services, coordinating shipments and overseeing delivery processes in Africa. The core functions and industries of these two companies are quite different, making them not comparable for transfer pricing purposes. Additionally, the website was inaccessible, which limits the information available for comparison.</t>
+Reasoning:
+The company under review, ALB - AREA LOGISTICA DA BOBADELA, S.A., specializes in warehouse management and distribution services, while the tested party in the medical industry focuses on procurement, logistics coordination, and delivery processes in Africa. The differences in core functions and industries suggest that they are not directly comparable for transfer pricing purposes. Additionally, the lack of access to the company's website further limits the ability to assess its operations and compare them to the tested party.</t>
         </is>
       </c>
     </row>
@@ -543,8 +544,8 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Not Comparable 
-The company under review, ALBERTS LOGISTIK GMBH &amp; CO. KG, is primarily focused on providing transportation, warehousing, and inventory management services in the region, catering to manufacturers, distributors, and retailers. On the other hand, the tested party is a procurement and logistics service provider in the medical industry in the Netherlands, with a focus on coordinating shipments, handling local storage, and overseeing delivery processes in Africa. There are significant differences in the core functions, industry focus, and geographic scope between the two companies, making them not comparable for transfer pricing purposes.</t>
+          <t>Not Comparable
+While both companies are involved in logistics and transportation services, the tested party specifically operates in the medical industry in Africa, with a focus on procurement and storage. On the other hand, the company under review, ALBERTS LOGISTIK GMBH &amp; CO. KG, appears to be more focused on providing transportation, warehousing, and inventory management services to manufacturers, distributors, and retailers. The industries, core functions, and target markets of the two companies are different, making them not directly comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -571,7 +572,8 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>Comparable
-Both companies provide logistics services within their respective industries, focusing on coordination, storage, and transportation of goods. While the tested party operates in the medical industry and the company under review operates in the automotive industry, the core functions and services offered by both companies are similar enough to be considered comparable for transfer pricing purposes.</t>
+Reasoning:
+Both companies provide logistics services targeting specific industries (medical and automotive), focusing on distribution, storage, and coordination of shipments. They also both serve as intermediaries in their respective industries, managing processes and operations for their clients. The nature of their services and client base makes them comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -597,8 +599,9 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Comparable.
-Both companies are involved in providing logistics and shipping-related services, with a focus on coordinating shipments and overseeing delivery processes. While the industries may differ slightly, the core functions and services offered by both companies are similar enough to be considered comparable for transfer pricing purposes.</t>
+          <t>Not Comparable.
+The company under review, ALFA SHIPPING AGENCY SRL, specializes in shipping and maritime logistics services, such as port agency services and cargo handling. Their primary focus seems to be on facilitating the movement of goods through maritime transport. On the other hand, the tested party in the medical industry in the Netherlands is involved in procurement and logistics services, specific to the medical industry in Africa.
+Therefore, these two companies operate in entirely different industries and provide different services, making them not comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -615,7 +618,7 @@
 Description: This company specializes in providing tailored products and services across various sectors, catering primarily to local and regional customers
 Website: WWW.ALMEIDAPESTANA.PT
 Website Content Extracted:
- Error accessing website: http://WWW.ALMEIDAPESTANA.PT – HTTPConnectionPool(host='www.almeidapestana.pt', port=80): Max retries exceeded with url: / (Caused by NameResolutionError("&lt;urllib3.connection.HTTPConnection object at 0x7f617cbff3d0&gt;: Failed to resolve 'www.almeidapestana.pt' ([Errno -2] Name or service not known)"))
+ Error accessing website: http://WWW.ALMEIDAPESTANA.PT – HTTPConnectionPool(host='www.almeidapestana.pt', port=80): Max retries exceeded with url: / (Caused by NameResolutionError("&lt;urllib3.connection.HTTPConnection object at 0x7efd71726ad0&gt;: Failed to resolve 'www.almeidapestana.pt' ([Errno -2] Name or service not known)"))
 Question:
 Based on the business description, website content and the tested party’s functions, is this company comparable for transfer pricing purposes? 
 Please answer with "Comparable" or "Not Comparable", and explain your reasoning briefly.
@@ -625,8 +628,7 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>Not Comparable.
-Reasoning:
-The company under review, ALMEIDA &amp; PESTANA, LDA, operates in the transportation services industry in Portugal, providing tailored products and services to local and regional customers. This is different from the tested party, a procurement and logistics service provider in the medical industry in the Netherlands. The core functions and industries of the two companies are not sufficiently similar to be considered comparable for transfer pricing purposes.</t>
+The company under review, ALMEIDA &amp; PESTANA, LDA, operates in the transportation services sector, while the tested party functions in the medical procurement and logistics services industry. Their core functions and target markets are different, making them not directly comparable for transfer pricing purposes. Additionally, the inability to access the company's website makes it difficult to gather more detailed information for a thorough comparison.</t>
         </is>
       </c>
     </row>
@@ -654,7 +656,7 @@
         <is>
           <t>Not Comparable
 Reasoning:
-The company under review, ALOG LTD OOD, operates in the transportation industry in Bulgaria, offering services such as automotive transport, air transport, sea transport, and warehouse logistics. The tested party is a procurement and logistics service provider in the medical industry in the Netherlands, focused on coordinating shipments, handling local storage, and overseeing delivery processes in Africa. The industries, functions, and geographic locations of the two companies are significantly different, making them not comparable for transfer pricing purposes.</t>
+The description of ALOG LTD OOD indicates that it operates in the transportation services industry, while the tested party is a procurement and logistics service provider in the medical industry. The core functions of the tested party involve coordinating shipments, handling local storage, and overseeing delivery processes in Africa, which is different from the services offered by ALOG LTD OOD. Additionally, the website content of ALOG LTD OOD does not provide enough information to determine if the company is comparable in terms of size, market, or functions to the tested party.</t>
         </is>
       </c>
     </row>
@@ -680,8 +682,9 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Not Comparable.
-The company under review, AUTOTALLERES GUTIERREZ SL, specializes in automobile repair and maintenance services, while the tested party is a procurement and logistics service provider in the medical industry. These two companies operate in completely different industries and have different core functions, making them not comparable for transfer pricing purposes.</t>
+          <t>Not Comparable
+Reasoning:
+The company under review, AUTOTALLERES GUTIERREZ SL, specializes in automobile repair and maintenance services, while the tested party is a procurement and logistics service provider in the medical industry. The nature of their core functions, customer base, and industry focus differ significantly, making them not comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -708,7 +711,8 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>Not Comparable.
-While both companies operate in the logistics industry, the tested party specifically focuses on procurement and logistics services in the medical industry in Africa, while the company under review offers a wider range of logistics services in Greece. The differences in geographic focus, industry specialization, and core functions indicate that these companies may not be directly comparable for transfer pricing purposes.</t>
+Reasoning:
+The tested party is a Netherlands-based procurement and logistics service provider in the medical industry focusing on shipments, storage, and delivery processes in Africa. The company under review, B.T.L. TRANSPORT LOGISTICS S.A., is a Greece-based logistics company specializing in freight transportation, warehousing, and supply chain management solutions. While both companies operate in the logistics industry, they serve different markets (medical industry vs general transportation services) and offer different core functions. These differences could result in significant variations in business models, risk profiles, and profit potential, making them not comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -734,8 +738,9 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Not Comparable.
-Reasoning: The tested party is a procurement and logistics service provider in the medical industry, while the company under review focuses on providing management and administrative services in the transportation industry. The differences in core functions and industries make these companies not comparable for transfer pricing purposes.</t>
+          <t>Not Comparable
+Reasoning:
+The tested party is a procurement and logistics service provider in the medical industry, focusing on coordinating shipments and overseeing delivery processes in Africa. On the other hand, the company under review, BARBIERI GESTIONI SRL, provides management and administrative services in the transportation industry in Italy. The core functions and industries of the two companies are quite different, thus making them not comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -761,9 +766,8 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Not Comparable
-Reasoning:
-The limited information available about BARTRANSIS UAB, coupled with the lack of website content, makes it difficult to assess if this company is truly comparable for transfer pricing purposes. Additionally, the specific industry focus and core functions of the tested party in the medical procurement and logistics sector may not align with the transportation services sector that BARTRANSIS UAB operates in. Without more detailed information, it is challenging to determine if the two companies are truly comparable.</t>
+          <t>Not Comparable. 
+The lack of specific information about the services provided by BARTRANSIS UAB on their website makes it difficult to assess if they are comparable to the Netherlands-based procurement and logistics service provider in the medical industry. Additionally, the possible regional or international customer base and diverse sector focus of BARTRANSIS UAB may indicate a different business model and market positioning compared to the tested party.</t>
         </is>
       </c>
     </row>
@@ -790,7 +794,7 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>Not Comparable.
-The company under review, BELLANDI SRL, operates in the retail-boats and marine supplies industry, specifically in water transportation services. Their core business activities do not align with the procurement and logistics services provided by the tested party in the medical industry. Additionally, the geographical focus and customer base of the two companies differ significantly. As a result, they are not comparable for transfer pricing purposes.</t>
+The company under review, BELLANDI SRL, operates in the retail-boats and marine supplies industry in Italy, specifically as a dealer for BENETEAU boats. On the other hand, the tested party is a procurement and logistics service provider in the medical industry based in the Netherlands. The core functions and industries of these two companies are different, making them not comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -817,7 +821,8 @@
       <c r="B15" t="inlineStr">
         <is>
           <t>Not Comparable.
-While both companies operate in the logistics industry, the core functions and services offered are quite different. The tested party mainly focuses on procurement and logistics services in the medical industry in Africa, while the company under review in Greece specializes in logistics and transportation services, including freight forwarding and customs brokerage. The differences in core functions and target markets make these two companies not comparable for transfer pricing purposes.</t>
+While both companies are involved in logistics and transportation services, the core functions and operations of the two companies differ significantly. The tested party in the medical industry focuses on procurement and logistics services specifically in Africa, whereas the company under review, BEST LOGISTICS NORTH S.A., offers a wide range of logistics services in Greece.
+The geographical focus, industry specialization, and core services provided by the two companies are not aligned, making them not directly comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>
@@ -843,8 +848,8 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Not Comparable
-While both companies operate within the logistics and transportation sector, there are significant differences in their core functions and geographical focus. The tested party is specifically focused on procurement and logistics services in the medical industry in Africa, while the company under review operates in Hungary and offers a range of transportation services. The differing industry focuses and geographical regions make these companies not directly comparable for transfer pricing purposes.</t>
+          <t>Not Comparable.
+The tested party is specifically focused on providing procurement and logistics services in the medical industry in Africa, while the company under review operates within the broader logistics and transportation sector in Hungary. The differences in industry focus and geographical market may result in significant differences in business operations, risks undertaken, and pricing strategies, making them not directly comparable for transfer pricing purposes.</t>
         </is>
       </c>
     </row>

</xml_diff>